<commit_message>
removed singel age group
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="4160" yWindow="3280" windowWidth="26240" windowHeight="16440" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-25600" yWindow="-3920" windowWidth="25600" windowHeight="21000" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Innstillinger" sheetId="1" state="visible" r:id="rId1"/>
@@ -19,18 +19,12 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <sz val="8"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -495,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="12.33203125" bestFit="1" customWidth="1" min="2" max="2"/>
@@ -518,6 +512,16 @@
           <t>round_length_minutes</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>deltakelser_per_lag_før_jul</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>deltakelser_per_lag_etter_jul</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -531,6 +535,12 @@
       <c r="C2" t="n">
         <v>15</v>
       </c>
+      <c r="D2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -544,58 +554,88 @@
       <c r="C3" t="n">
         <v>15</v>
       </c>
+      <c r="D3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>U9</t>
+          <t>JU8</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C4" t="n">
         <v>15</v>
       </c>
+      <c r="D4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>U10</t>
+          <t>U9</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C5" t="n">
         <v>15</v>
       </c>
+      <c r="D5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>JU9</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C6" t="n">
         <v>15</v>
       </c>
+      <c r="D6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>U12</t>
+          <t>U10</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C7" t="n">
         <v>15</v>
       </c>
+      <c r="D7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -609,31 +649,87 @@
       <c r="C8" t="n">
         <v>15</v>
       </c>
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>JU11</t>
+          <t>U11</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C9" t="n">
         <v>15</v>
       </c>
+      <c r="D9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>JU12</t>
+          <t>JU11</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C10" t="n">
         <v>15</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>U12</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>2</v>
+      </c>
+      <c r="C11" t="n">
+        <v>15</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>JU12</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" t="n">
+        <v>15</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove roster region and skill metadata
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-25600" yWindow="-3920" windowWidth="25600" windowHeight="21000" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-25600" yWindow="-3920" windowWidth="25600" windowHeight="21000" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Innstillinger" sheetId="1" state="visible" r:id="rId1"/>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="12.33203125" bestFit="1" customWidth="1" min="2" max="2"/>
@@ -533,13 +533,13 @@
         <v>4</v>
       </c>
       <c r="C2" t="n">
-        <v>15</v>
+        <v>120</v>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -552,13 +552,13 @@
         <v>4</v>
       </c>
       <c r="C3" t="n">
-        <v>15</v>
+        <v>120</v>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -571,13 +571,13 @@
         <v>4</v>
       </c>
       <c r="C4" t="n">
-        <v>15</v>
+        <v>120</v>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -590,146 +590,108 @@
         <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>15</v>
+        <v>120</v>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>JU9</t>
+          <t>U10</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>3</v>
       </c>
       <c r="C6" t="n">
-        <v>15</v>
+        <v>105</v>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>U10</t>
+          <t>JU10</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>3</v>
       </c>
       <c r="C7" t="n">
-        <v>15</v>
+        <v>105</v>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>JU10</t>
+          <t>U11</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>3</v>
       </c>
       <c r="C8" t="n">
-        <v>15</v>
+        <v>105</v>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U12</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C9" t="n">
-        <v>15</v>
+        <v>75</v>
       </c>
       <c r="D9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>JU11</t>
+          <t>JU12</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C10" t="n">
-        <v>15</v>
+        <v>75</v>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E10" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>U12</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>2</v>
-      </c>
-      <c r="C11" t="n">
-        <v>15</v>
-      </c>
-      <c r="D11" t="n">
-        <v>2</v>
-      </c>
-      <c r="E11" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>JU12</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>2</v>
-      </c>
-      <c r="C12" t="n">
-        <v>15</v>
-      </c>
-      <c r="D12" t="n">
-        <v>2</v>
-      </c>
-      <c r="E12" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -743,7 +705,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E71"/>
+  <dimension ref="A1:C68"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="9.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -769,16 +731,6 @@
           <t>age_group</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>region</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>skill_level</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -980,24 +932,24 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>JU11</t>
+          <t>JU12</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Frisk Asker</t>
+          <t>Holmen</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Frisk Asker</t>
+          <t>Holmen</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>JU12</t>
+          <t>U7</t>
         </is>
       </c>
     </row>
@@ -1014,7 +966,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>U7</t>
+          <t>U8</t>
         </is>
       </c>
     </row>
@@ -1031,7 +983,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>U8</t>
+          <t>U9</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1000,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>U9</t>
+          <t>U10</t>
         </is>
       </c>
     </row>
@@ -1065,7 +1017,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>U10</t>
+          <t>U11</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1034,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U12</t>
         </is>
       </c>
     </row>
@@ -1099,11 +1051,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>U12</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
+          <t>JU10</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" collapsed="1">
       <c r="A21" t="inlineStr">
         <is>
           <t>Holmen</t>
@@ -1116,41 +1068,41 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>JU10</t>
+          <t>JU12</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Holmen</t>
+          <t>Jar</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Holmen</t>
+          <t>Jar 1</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>JU11</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" collapsed="1">
+          <t>U7</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Holmen</t>
+          <t>Jar</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Holmen</t>
+          <t>Jar 1</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>JU12</t>
+          <t>U8</t>
         </is>
       </c>
     </row>
@@ -1167,7 +1119,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>U7</t>
+          <t>U9</t>
         </is>
       </c>
     </row>
@@ -1179,12 +1131,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Jar 1</t>
+          <t>Jar 2</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>U8</t>
+          <t>U9</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1153,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>U9</t>
+          <t>U10</t>
         </is>
       </c>
     </row>
@@ -1218,7 +1170,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>U9</t>
+          <t>U10</t>
         </is>
       </c>
     </row>
@@ -1230,7 +1182,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Jar 1</t>
+          <t>Jar 3</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1247,7 +1199,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Jar 2</t>
+          <t>Jar 4</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1264,12 +1216,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Jar 3</t>
+          <t>Jar 1</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>U10</t>
+          <t>U11</t>
         </is>
       </c>
     </row>
@@ -1281,12 +1233,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Jar 4</t>
+          <t>Jar 2</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>U10</t>
+          <t>U11</t>
         </is>
       </c>
     </row>
@@ -1298,7 +1250,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Jar 1</t>
+          <t>Jar 3</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1315,12 +1267,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Jar 2</t>
+          <t>Jar 1</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U12</t>
         </is>
       </c>
     </row>
@@ -1332,12 +1284,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Jar 3</t>
+          <t>Jar 2</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U12</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1301,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Jar 1</t>
+          <t>Jar 3</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1366,12 +1318,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Jar 2</t>
+          <t>Jar 1</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>U12</t>
+          <t>JU10</t>
         </is>
       </c>
     </row>
@@ -1383,63 +1335,63 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Jar 3</t>
+          <t>Jar 1</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>U12</t>
+          <t>JU12</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Jutul</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Jar 1</t>
+          <t>Jutul</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>JU10</t>
+          <t>U7</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Jutul</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Jar 1</t>
+          <t>Jutul</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>JU11</t>
+          <t>U8</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Jutul</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Jar 1</t>
+          <t>Jutul</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>JU12</t>
+          <t>U9</t>
         </is>
       </c>
     </row>
@@ -1456,7 +1408,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>U7</t>
+          <t>U10</t>
         </is>
       </c>
     </row>
@@ -1473,7 +1425,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>U8</t>
+          <t>U11</t>
         </is>
       </c>
     </row>
@@ -1490,7 +1442,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>U9</t>
+          <t>U12</t>
         </is>
       </c>
     </row>
@@ -1507,58 +1459,58 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>U10</t>
+          <t>JU10</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Jutul</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Jutul</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U7</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Jutul</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Jutul</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>U12</t>
+          <t>U8</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Jutul</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Jutul</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>JU10</t>
+          <t>U9</t>
         </is>
       </c>
     </row>
@@ -1575,7 +1527,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>U7</t>
+          <t>U10</t>
         </is>
       </c>
     </row>
@@ -1592,7 +1544,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>U8</t>
+          <t>U11</t>
         </is>
       </c>
     </row>
@@ -1609,7 +1561,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>U9</t>
+          <t>U12</t>
         </is>
       </c>
     </row>
@@ -1626,7 +1578,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>U10</t>
+          <t>JU10</t>
         </is>
       </c>
     </row>
@@ -1643,7 +1595,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>JU11</t>
         </is>
       </c>
     </row>
@@ -1660,58 +1612,58 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>U12</t>
+          <t>JU12</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Ringerike</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Ringerike</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>JU10</t>
+          <t>U9</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Ringerike</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Ringerike</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>JU11</t>
+          <t>U10</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Ringerike</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Ringerike 1</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>JU12</t>
+          <t>U11</t>
         </is>
       </c>
     </row>
@@ -1723,24 +1675,24 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Ringerike</t>
+          <t>Ringerike 2</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>U9</t>
+          <t>U11</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Ringerike</t>
+          <t>Sandefjord</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Ringerike</t>
+          <t>Sandefjord</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1752,12 +1704,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Ringerike</t>
+          <t>Sandefjord</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Ringerike 1</t>
+          <t>Sandefjord</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -1769,85 +1721,85 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Ringerike</t>
+          <t>Skien</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Ringerike 2</t>
+          <t>Skien</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U10</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Sandefjord</t>
+          <t>Skien</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Sandefjord</t>
+          <t>Skien</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>U10</t>
+          <t>U11</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Sandefjord</t>
+          <t>Tønsberg</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Sandefjord</t>
+          <t>Tønsberg</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U7</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Skien</t>
+          <t>Tønsberg</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Skien</t>
+          <t>Tønsberg</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>U10</t>
+          <t>U8</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Skien</t>
+          <t>Tønsberg</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Skien</t>
+          <t>Tønsberg</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U9</t>
         </is>
       </c>
     </row>
@@ -1859,12 +1811,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Tønsberg</t>
+          <t>Tønsberg 2</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>U7</t>
+          <t>U10</t>
         </is>
       </c>
     </row>
@@ -1881,7 +1833,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>U8</t>
+          <t>U10</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1850,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>U9</t>
+          <t>U11</t>
         </is>
       </c>
     </row>
@@ -1910,61 +1862,10 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Tønsberg 2</t>
+          <t>Tønsberg</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
-        <is>
-          <t>U10</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>Tønsberg</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>Tønsberg</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>U10</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>Tønsberg</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>Tønsberg</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>U11</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>Tønsberg</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>Tønsberg</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
         <is>
           <t>U12</t>
         </is>

</xml_diff>

<commit_message>
added previous season + updated input-xlsx based on that
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -705,7 +705,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C68"/>
+  <dimension ref="A1:C128"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="9.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -740,7 +740,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Frisk Asker</t>
+          <t>Frisk Asker 1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -757,12 +757,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Frisk Asker</t>
+          <t>Frisk Asker 2</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>U8</t>
+          <t>U7</t>
         </is>
       </c>
     </row>
@@ -774,12 +774,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Frisk Asker 1</t>
+          <t>Frisk Asker 3</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>U9</t>
+          <t>U7</t>
         </is>
       </c>
     </row>
@@ -791,12 +791,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Frisk Asker 2</t>
+          <t>Frisk Asker 1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>U9</t>
+          <t>U8</t>
         </is>
       </c>
     </row>
@@ -808,12 +808,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Frisk Asker 1</t>
+          <t>Frisk Asker 2</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>U10</t>
+          <t>U8</t>
         </is>
       </c>
     </row>
@@ -825,12 +825,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Frisk Asker 2</t>
+          <t>Frisk Asker 3</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>U10</t>
+          <t>U8</t>
         </is>
       </c>
     </row>
@@ -842,12 +842,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Frisk Asker 3</t>
+          <t>Frisk Asker</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>U10</t>
+          <t>JU8</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U9</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U9</t>
         </is>
       </c>
     </row>
@@ -893,12 +893,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Frisk Asker</t>
+          <t>Frisk Asker 3</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>U12</t>
+          <t>U9</t>
         </is>
       </c>
     </row>
@@ -910,12 +910,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Frisk Asker</t>
+          <t>Frisk Asker 4</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>JU10</t>
+          <t>U9</t>
         </is>
       </c>
     </row>
@@ -927,75 +927,75 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Frisk Asker</t>
+          <t>Frisk Asker 5</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>JU12</t>
+          <t>U9</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Holmen</t>
+          <t>Frisk Asker</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Holmen</t>
+          <t>Frisk Asker 1</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>U7</t>
+          <t>U10</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Holmen</t>
+          <t>Frisk Asker</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Holmen</t>
+          <t>Frisk Asker 2</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>U8</t>
+          <t>U10</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Holmen</t>
+          <t>Frisk Asker</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Holmen</t>
+          <t>Frisk Asker 3</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>U9</t>
+          <t>U10</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Holmen</t>
+          <t>Frisk Asker</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Holmen</t>
+          <t>Frisk Asker 4</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1007,420 +1007,420 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Holmen</t>
+          <t>Frisk Asker</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Holmen</t>
+          <t>Frisk Asker 1</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>JU10</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Holmen</t>
+          <t>Frisk Asker</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Holmen</t>
+          <t>Frisk Asker 2</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>U12</t>
+          <t>JU10</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Holmen</t>
+          <t>Frisk Asker</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Holmen</t>
+          <t>Frisk Asker 1</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>JU10</t>
+          <t>U11</t>
         </is>
       </c>
     </row>
     <row r="21" collapsed="1">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Holmen</t>
+          <t>Frisk Asker</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Holmen</t>
+          <t>Frisk Asker 2</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>JU12</t>
+          <t>U11</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Frisk Asker</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Jar 1</t>
+          <t>Frisk Asker 3</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>U7</t>
+          <t>U11</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Frisk Asker</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Jar 1</t>
+          <t>Frisk Asker 1</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>U8</t>
+          <t>U12</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Frisk Asker</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Jar 1</t>
+          <t>Frisk Asker 2</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>U9</t>
+          <t>U12</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Frisk Asker</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Jar 2</t>
+          <t>Frisk Asker 3</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>U9</t>
+          <t>U12</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Frisk Asker</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Jar 1</t>
+          <t>Frisk Asker 4</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>U10</t>
+          <t>U12</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Frisk Asker</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Jar 2</t>
+          <t>Frisk Asker 5</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>U10</t>
+          <t>U12</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Frisk Asker</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Jar 3</t>
+          <t>Frisk Asker</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>U10</t>
+          <t>JU12</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Holmen</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Jar 4</t>
+          <t>Holmen 1</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>U10</t>
+          <t>U7</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Holmen</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Jar 1</t>
+          <t>Holmen 2</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U7</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Holmen</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Jar 2</t>
+          <t>Holmen 1</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U8</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Holmen</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Jar 3</t>
+          <t>Holmen 2</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U8</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Holmen</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Jar 1</t>
+          <t>Holmen 3</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>U12</t>
+          <t>U8</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Holmen</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Jar 2</t>
+          <t>Holmen</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>U12</t>
+          <t>JU8</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Holmen</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Jar 3</t>
+          <t>Holmen 1</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>U12</t>
+          <t>U9</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Holmen</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Jar 1</t>
+          <t>Holmen 2</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>JU10</t>
+          <t>U9</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Holmen</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Jar 1</t>
+          <t>Holmen 3</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>JU12</t>
+          <t>U9</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Jutul</t>
+          <t>Holmen</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Jutul</t>
+          <t>Holmen 4</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>U7</t>
+          <t>U9</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Jutul</t>
+          <t>Holmen</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Jutul</t>
+          <t>Holmen 1</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>U8</t>
+          <t>U10</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Jutul</t>
+          <t>Holmen</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Jutul</t>
+          <t>Holmen 2</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>U9</t>
+          <t>U10</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Jutul</t>
+          <t>Holmen</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Jutul</t>
+          <t>Holmen 1</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>U10</t>
+          <t>U11</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Jutul</t>
+          <t>Holmen</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Jutul</t>
+          <t>Holmen 2</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1432,46 +1432,46 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Jutul</t>
+          <t>Jar</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Jutul</t>
+          <t>Jar 1</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>U12</t>
+          <t>U7</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Jutul</t>
+          <t>Jar</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Jutul</t>
+          <t>Jar 2</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>JU10</t>
+          <t>U7</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Jar</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Jar 3</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1483,148 +1483,148 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Jar</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Jar 4</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>U8</t>
+          <t>U7</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Jar</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Jar 1</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>U9</t>
+          <t>U8</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Jar</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Jar 2</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>U10</t>
+          <t>U8</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Jar</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Jar 3</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U8</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Jar</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Jar 4</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>U12</t>
+          <t>U8</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Jar</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Jar</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>JU10</t>
+          <t>JU8</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Jar</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Jar 1</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>JU11</t>
+          <t>U9</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Jar</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Jar 2</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>JU12</t>
+          <t>U9</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Ringerike</t>
+          <t>Jar</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Ringerike</t>
+          <t>Jar 3</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1636,63 +1636,63 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Ringerike</t>
+          <t>Jar</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Ringerike</t>
+          <t>Jar 4</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>U10</t>
+          <t>U9</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Ringerike</t>
+          <t>Jar</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Ringerike 1</t>
+          <t>Jar 5</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U9</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Ringerike</t>
+          <t>Jar</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Ringerike 2</t>
+          <t>Jar 6</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U9</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Sandefjord</t>
+          <t>Jar</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Sandefjord</t>
+          <t>Jar 1</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1704,29 +1704,29 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Sandefjord</t>
+          <t>Jar</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Sandefjord</t>
+          <t>Jar 2</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U10</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Skien</t>
+          <t>Jar</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Skien</t>
+          <t>Jar 3</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -1738,114 +1738,114 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Skien</t>
+          <t>Jar</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Skien</t>
+          <t>Jar 4</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U10</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Tønsberg</t>
+          <t>Jar</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Tønsberg</t>
+          <t>Jar 5</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>U7</t>
+          <t>U10</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Tønsberg</t>
+          <t>Jar</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Tønsberg</t>
+          <t>Jar 6</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>U8</t>
+          <t>U10</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Tønsberg</t>
+          <t>Jar</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Tønsberg</t>
+          <t>Jar 7</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>U9</t>
+          <t>U10</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Tønsberg</t>
+          <t>Jar</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Tønsberg 2</t>
+          <t>Jar 1</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>U10</t>
+          <t>U11</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Tønsberg</t>
+          <t>Jar</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Tønsberg</t>
+          <t>Jar 2</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>U10</t>
+          <t>U11</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Tønsberg</t>
+          <t>Jar</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Tønsberg</t>
+          <t>Jar 3</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -1857,17 +1857,1037 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
+          <t>Jar</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Jar 4</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>U11</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Jar</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Jar 1</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>U12</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Jar</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Jar 2</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>U12</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Jar</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Jar 3</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>U12</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Jar</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Jar 4</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>U12</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Jutul</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Jutul 1</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>U7</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Jutul</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Jutul 2</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>U7</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Jutul</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Jutul 1</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>U8</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Jutul</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Jutul 2</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>U8</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Jutul</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Jutul 3</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>U8</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Jutul</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Jutul</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>JU8</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Jutul</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Jutul 1</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>U9</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Jutul</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Jutul 2</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>U9</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Jutul</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Jutul 3</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>U9</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Jutul</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Jutul 1</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>U10</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Jutul</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Jutul 2</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>U10</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Jutul</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Jutul 1</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>U11</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Jutul</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Jutul 2</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>U11</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Jutul</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Jutul 3</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>U11</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Jutul</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Jutul 1</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>U12</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Jutul</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Jutul 2</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>U12</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Kongsberg</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Kongsberg</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>U7</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Kongsberg</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Kongsberg</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>U8</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Kongsberg</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Kongsberg</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>U9</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Kongsberg</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Kongsberg</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>U10</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Kongsberg</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Kongsberg</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>JU12</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Ringerike</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Ringerike 1</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>U8</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Ringerike</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Ringerike 2</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>U8</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Ringerike</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Ringerike</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>JU8</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Ringerike</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Ringerike 1</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>U9</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Ringerike</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Ringerike 2</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>U9</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Ringerike</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Ringerike 3</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>U9</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Ringerike</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Ringerike 1</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>U10</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Ringerike</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Ringerike 2</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>U10</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Ringerike</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Ringerike</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>JU10</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Ringerike</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Ringerike 1</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>U11</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Ringerike</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Ringerike 2</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>U11</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Ringerike</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Ringerike 1</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>U12</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Ringerike</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Ringerike 2</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>U12</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Ringerike</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Ringerike 1</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>JU12</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Ringerike</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Ringerike 2</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>JU12</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Sandefjord</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Sandefjord</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>U7</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Sandefjord</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Sandefjord</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>U8</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Sandefjord</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Sandefjord</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>U10</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Skien</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Skien</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>U7</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Skien</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Skien</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>U8</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Skien</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Skien</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>JU8</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Skien</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Skien</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>U10</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Skien</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Skien</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>JU10</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Skien</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Skien</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>JU12</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
           <t>Tønsberg</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
+      <c r="B118" t="inlineStr">
         <is>
           <t>Tønsberg</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr">
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>U7</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Tønsberg</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Tønsberg</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>U8</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Tønsberg</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Tønsberg</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>U9</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Tønsberg</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Tønsberg 1</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>U10</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Tønsberg</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Tønsberg 2</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>U10</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Tønsberg</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Tønsberg 1</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>U11</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Tønsberg</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Tønsberg 2</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>U11</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Tønsberg</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Tønsberg</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
         <is>
           <t>U12</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Tønsberg</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Tønsberg</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>JU12</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Jar/Jutul</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Jar/Jutul</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>JU10</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Jar/Jutul</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Jar/Jutul</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>JU12</t>
         </is>
       </c>
     </row>

</xml_diff>